<commit_message>
Update model performance xlsx and add DeLong heatmap outputs; ignore EJP/Frontiers/Manuscript folders
</commit_message>
<xml_diff>
--- a/06_Modelling/06d_影像+临床_mRMR_10调参_noSMOTE-LGBM0.7568最终版/04_Model_Performance.xlsx
+++ b/06_Modelling/06d_影像+临床_mRMR_10调参_noSMOTE-LGBM0.7568最终版/04_Model_Performance.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Softwares\PycharmProject\Radiomics\06_Modelling\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Softwares\PycharmProject\Radiomics\06_Modelling\06d_影像+临床_mRMR_10调参_noSMOTE-LGBM0.7568最终版\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC74B5E-7401-4EE8-B29A-9537A1E8CA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4A6E590-14EC-4EDE-B39E-A352C2A95730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4520" yWindow="2820" windowWidth="16280" windowHeight="10327" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6690" yWindow="6697" windowWidth="21600" windowHeight="11333" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -105,9 +105,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="177" formatCode="0.0000"/>
+    <numFmt numFmtId="176" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,6 +123,15 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
@@ -164,12 +173,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -473,9 +483,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R10"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,7 +538,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -556,7 +566,7 @@
       <c r="I2" s="2">
         <v>0.6737967914438503</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="3">
         <v>0.72773809523809518</v>
       </c>
       <c r="K2" s="2">
@@ -584,7 +594,7 @@
         <v>0.79722381875020365</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -612,7 +622,7 @@
       <c r="I3" s="2">
         <v>0.6470588235294118</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="3">
         <v>0.6713690476190477</v>
       </c>
       <c r="K3" s="2">
@@ -640,7 +650,7 @@
         <v>0.74365032851375834</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -668,7 +678,7 @@
       <c r="I4" s="2">
         <v>0.66310160427807485</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="3">
         <v>0.74023809523809514</v>
       </c>
       <c r="K4" s="2">
@@ -696,7 +706,7 @@
         <v>0.80891248246728864</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -724,7 +734,7 @@
       <c r="I5" s="2">
         <v>0.68449197860962563</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="3">
         <v>0.75488095238095243</v>
       </c>
       <c r="K5" s="2">
@@ -752,7 +762,7 @@
         <v>0.82103722765482934</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -780,7 +790,7 @@
       <c r="I6" s="2">
         <v>0.64171122994652408</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="3">
         <v>0.73845238095238108</v>
       </c>
       <c r="K6" s="2">
@@ -808,7 +818,7 @@
         <v>0.80726604554865422</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
@@ -836,7 +846,7 @@
       <c r="I7" s="2">
         <v>0.69518716577540107</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="3">
         <v>0.73202380952380952</v>
       </c>
       <c r="K7" s="2">
@@ -864,7 +874,7 @@
         <v>0.79814032004821478</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
@@ -892,7 +902,7 @@
       <c r="I8" s="2">
         <v>0.70053475935828879</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="3">
         <v>0.75678571428571428</v>
       </c>
       <c r="K8" s="2">
@@ -920,7 +930,7 @@
         <v>0.82505676207036527</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -948,7 +958,7 @@
       <c r="I9" s="2">
         <v>0.62566844919786091</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="3">
         <v>0.66761904761904767</v>
       </c>
       <c r="K9" s="2">
@@ -976,7 +986,7 @@
         <v>0.74480453244597977</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -1004,7 +1014,7 @@
       <c r="I10" s="2">
         <v>0.62566844919786091</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="3">
         <v>0.66535714285714276</v>
       </c>
       <c r="K10" s="2">

</xml_diff>